<commit_message>
RESHIPPED (task130): round 1 restored by the author's decision after round 2 was sent back
Every task130 file back to 9bf3cbc ($784,000); round 2 ($587,000, the Early
Resolution Program's class experience) recorded in the design note, the card's
lineage, pipeline.json and the ledger's earlier architectures. Nine Three rules
lines from the 10/10 audit added true to round 1; precut.py 49 checks, 0 WARN.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task130/golden/trust_funding_2027.xlsx
+++ b/task130/golden/trust_funding_2027.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="96">
   <si>
     <t>Corvane Professional Liability Trust: 2027 contribution</t>
   </si>
@@ -34,10 +34,7 @@
     <t>2027 Contribution ($)</t>
   </si>
   <si>
-    <t>Expected number of Claims first made in 2027</t>
-  </si>
-  <si>
-    <t>What each Participating Entity pays (funding policy section 2: in proportion to its share of the 2027 exposure under 3.3)</t>
+    <t>By Participating Entity</t>
   </si>
   <si>
     <t>Participating Entity</t>
@@ -49,10 +46,10 @@
     <t>Covered FTE-years in the Trust, 2027</t>
   </si>
   <si>
-    <t>Share of exposure</t>
-  </si>
-  <si>
-    <t>Pays ($)</t>
+    <t>Expected Claims</t>
+  </si>
+  <si>
+    <t>Expected cost ($)</t>
   </si>
   <si>
     <t>Tolliver Falls Hospital</t>
@@ -82,7 +79,37 @@
     <t>All entities</t>
   </si>
   <si>
-    <t>Payments are each entity's share of the Contribution for the year, paid in equal quarterly instalments; shares follow the staffing plan's covered FTE-years from each Transition Date.</t>
+    <t>By specialty class</t>
+  </si>
+  <si>
+    <t>Specialty class</t>
+  </si>
+  <si>
+    <t>Obstetrics</t>
+  </si>
+  <si>
+    <t>Surgery</t>
+  </si>
+  <si>
+    <t>Emergency Medicine</t>
+  </si>
+  <si>
+    <t>Anesthesiology</t>
+  </si>
+  <si>
+    <t>Hospital and Medical Specialties</t>
+  </si>
+  <si>
+    <t>Primary Care</t>
+  </si>
+  <si>
+    <t>Advanced Practice</t>
+  </si>
+  <si>
+    <t>All classes</t>
+  </si>
+  <si>
+    <t>Brennick Community Hospital joins on 1 October 2027: three months of exposure, and only the Claims made by 31 December count.</t>
   </si>
   <si>
     <t>Source: risk management claims register extract valued 30 September 2026; legacy payroll 2017 to 2024; clinician staffing plan 2027, version 2026-09-29. Basis and definitions on the Notes sheet.</t>
@@ -184,34 +211,40 @@
     <t>Our reserves ($)</t>
   </si>
   <si>
-    <t>CL-2026-0049</t>
-  </si>
-  <si>
-    <t>IR-2026-00725</t>
-  </si>
-  <si>
-    <t>20 Jul 2026</t>
+    <t>CL-2026-0098</t>
+  </si>
+  <si>
+    <t>IR-2026-00613</t>
+  </si>
+  <si>
+    <t>23 Jun 2026</t>
   </si>
   <si>
     <t>Claim</t>
   </si>
   <si>
-    <t>CL-2026-0093</t>
-  </si>
-  <si>
-    <t>IR-2026-01310</t>
+    <t>CL-2026-0177</t>
+  </si>
+  <si>
+    <t>IR-2026-01269</t>
   </si>
   <si>
     <t>29 Sep 2026</t>
   </si>
   <si>
+    <t>CL-2026-0133</t>
+  </si>
+  <si>
+    <t>IR-2026-00734</t>
+  </si>
+  <si>
+    <t>28 Jul 2026</t>
+  </si>
+  <si>
     <t>Quillan Mutual's latest run is the one valued 30 September 2026 (issued 6 October 2026); revision 1 of its 30 June 2026 run, issued 9 October 2026, is an earlier valuation.</t>
   </si>
   <si>
-    <t>Claims that began as precautionary notices are carried on the runs under their notice numbers (RMN), which the notice log ties to the incident record opened at the notice; a suit that followed an earlier claim number for the same incident stays under that earlier number. Stoneleigh drops the punctuation from references.</t>
-  </si>
-  <si>
-    <t>Where a claim was registered under a new incident record rather than the one opened at its notice, the carrier's notice file is the same matter: the notice log's entity, event date and category match the register's claim, and the carrier holds it as a claim or suit. Notice files on claims against an entity alone are kept in the general liability register and match no claim here.</t>
+    <t>Claims that began as precautionary notices are carried on the runs under their notice numbers (RMN), which the notice log ties to incident numbers; a suit that followed an earlier claim number for the same incident stays under that earlier number. Stoneleigh drops the punctuation from references.</t>
   </si>
   <si>
     <t>Missing: open in the register at 30 September 2026 under the entity's coverage line, one per incident, with no record on the run. Reserves are the register's indemnity and defense reserves on our rows.</t>
@@ -223,7 +256,7 @@
     <t>Covered clinician FTE</t>
   </si>
   <si>
-    <t>One FTE per position held in September 2026, Schedule B jobs through the HCM job profile crosswalk, on the entity of the cost centre the position's lines are charged to. The HCM home entity on the extract is the worker's record when it ran in October: the clinicians who moved on 1 October 2026 carry their new entity on their September lines.</t>
+    <t>One FTE per position held in September 2026, Schedule B jobs through the HCM job profile crosswalk, on the entity of the cost centre the position's lines are charged to.</t>
   </si>
   <si>
     <t>Notes</t>
@@ -244,16 +277,10 @@
     <t>Each entity from its Transition Date (its Retroactive Date) to 31 December 2027: Claims made in 2027 from incidents on or after that date.</t>
   </si>
   <si>
-    <t>Claims handling</t>
-  </si>
-  <si>
-    <t>From its Transition Date every entity's patients can bring a request through the Early Resolution Program (Trust Agreement 5.2). Until now the Program has served Tolliver Falls and Alderwick only; Stoneleigh adjusted the medical group's and Brennick's claims, and none of their 69 experience Claims came through the Program. The Claims a first-year window can catch are mostly Program requests, so the 2027 window is costed on the experience generated under the Program: Tolliver Falls' and Alderwick's.</t>
-  </si>
-  <si>
     <t>Experience</t>
   </si>
   <si>
-    <t>The 123 Claims from incidents in 2017 to 2024 at Tolliver Falls and Alderwick naming Covered Clinicians, valued at paid plus case reserves on the Covered Clinicians' rows of the register extract valued 30 September 2026, trended at 5.0% a year from the incident year to 2027, against those hospitals' 2,655.2 covered FTE-years in the payroll for the same years, within each specialty class (funding policy 3.2 and 3.5); one rate for every entity (3.4).</t>
+    <t>The 328 Claims from incidents in 2017 to 2024 naming Covered Clinicians, valued at paid plus case reserves on the Covered Clinicians' rows of the register extract valued 30 September 2026, trended at 5.0% a year from the incident year to 2027, against 6,188.6 covered FTE-years in the payroll for the same years, pooled within each specialty class (funding policy 3.2 and 3.4).</t>
   </si>
   <si>
     <t>Exposure</t>
@@ -271,7 +298,7 @@
     <t>Not included</t>
   </si>
   <si>
-    <t>Administrative expenses, investment income, excess insurance and any margin (funding policy 3.6).</t>
+    <t>Administrative expenses, investment income, excess insurance and any margin (funding policy 3.5).</t>
   </si>
   <si>
     <t>Rounding</t>
@@ -290,9 +317,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -359,12 +385,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </xf>
@@ -377,19 +402,16 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -702,14 +724,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" customWidth="1"/>
     <col min="3" max="3" width="22.7109375" customWidth="1"/>
     <col min="4" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -727,130 +749,255 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>587000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+        <v>784000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4">
-        <v>10.2</v>
-      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="B7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
-        <v>5</v>
+      <c r="A8" t="s">
+        <v>9</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="C8" s="7">
+        <v>100.2</v>
+      </c>
+      <c r="D8" s="7">
+        <v>2.9</v>
+      </c>
+      <c r="E8" s="8">
+        <v>227000</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="8">
-        <v>113.4</v>
-      </c>
-      <c r="D9" s="9">
-        <v>0.1889567995554938</v>
-      </c>
-      <c r="E9" s="10">
-        <v>111000</v>
+      <c r="B9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="7">
+        <v>175.6</v>
+      </c>
+      <c r="D9" s="7">
+        <v>4.6</v>
+      </c>
+      <c r="E9" s="8">
+        <v>336000</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="8">
-        <v>205.5</v>
-      </c>
-      <c r="D10" s="9">
-        <v>0.3426170301430754</v>
-      </c>
-      <c r="E10" s="10">
-        <v>201000</v>
+      <c r="B10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="7">
+        <v>264.9</v>
+      </c>
+      <c r="D10" s="7">
+        <v>3.9</v>
+      </c>
+      <c r="E10" s="8">
+        <v>214000</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="8">
-        <v>265.4</v>
-      </c>
-      <c r="D11" s="9">
-        <v>0.4424503403250451</v>
-      </c>
-      <c r="E11" s="10">
-        <v>260000</v>
+      <c r="B11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="7">
+        <v>15.1</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="E11" s="8">
+        <v>7000</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="8">
-        <v>15.6</v>
-      </c>
-      <c r="D12" s="9">
-        <v>0.02597582997638561</v>
-      </c>
-      <c r="E12" s="10">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="B12" s="10"/>
+      <c r="C12" s="11">
+        <v>555.8</v>
+      </c>
+      <c r="D12" s="11">
+        <v>11.5</v>
+      </c>
+      <c r="E12" s="12">
+        <v>784000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="13">
-        <v>599.9</v>
-      </c>
-      <c r="D13" s="14">
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="13">
+        <v>30.7</v>
+      </c>
+      <c r="D16" s="13">
+        <v>2</v>
+      </c>
+      <c r="E16" s="14">
+        <v>148000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="13">
+        <v>61.7</v>
+      </c>
+      <c r="D17" s="13">
+        <v>2.3</v>
+      </c>
+      <c r="E17" s="14">
+        <v>291000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="13">
+        <v>43.7</v>
+      </c>
+      <c r="D18" s="13">
+        <v>2</v>
+      </c>
+      <c r="E18" s="14">
+        <v>68000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="13">
+        <v>26.7</v>
+      </c>
+      <c r="D19" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="E19" s="14">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="13">
+        <v>114.9</v>
+      </c>
+      <c r="D20" s="13">
+        <v>2.3</v>
+      </c>
+      <c r="E20" s="14">
+        <v>124000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="C21" s="13">
+        <v>108.4</v>
+      </c>
+      <c r="D21" s="13">
+        <v>1.4</v>
+      </c>
+      <c r="E21" s="14">
+        <v>26000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" s="13">
+        <v>169.6</v>
+      </c>
+      <c r="D22" s="13">
         <v>1</v>
       </c>
-      <c r="E13" s="15">
-        <v>587000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>20</v>
+      <c r="E22" s="14">
+        <v>62000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="10"/>
+      <c r="C23" s="11">
+        <v>555.8</v>
+      </c>
+      <c r="D23" s="11">
+        <v>11.5</v>
+      </c>
+      <c r="E23" s="12">
+        <v>784000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -877,292 +1024,292 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>18</v>
+      <c r="A3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="17">
-        <v>1000</v>
-      </c>
-      <c r="C4" s="17">
-        <v>0</v>
-      </c>
-      <c r="D4" s="17">
-        <v>0</v>
-      </c>
-      <c r="E4" s="17">
-        <v>0</v>
-      </c>
-      <c r="F4" s="17">
-        <v>1000</v>
+        <v>32</v>
+      </c>
+      <c r="B4" s="14">
+        <v>0</v>
+      </c>
+      <c r="C4" s="14">
+        <v>0</v>
+      </c>
+      <c r="D4" s="14">
+        <v>0</v>
+      </c>
+      <c r="E4" s="14">
+        <v>0</v>
+      </c>
+      <c r="F4" s="14">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="17">
-        <v>2000</v>
-      </c>
-      <c r="C5" s="17">
-        <v>0</v>
-      </c>
-      <c r="D5" s="17">
-        <v>0</v>
-      </c>
-      <c r="E5" s="17">
-        <v>0</v>
-      </c>
-      <c r="F5" s="17">
-        <v>2000</v>
+        <v>33</v>
+      </c>
+      <c r="B5" s="14">
+        <v>3000</v>
+      </c>
+      <c r="C5" s="14">
+        <v>0</v>
+      </c>
+      <c r="D5" s="14">
+        <v>0</v>
+      </c>
+      <c r="E5" s="14">
+        <v>0</v>
+      </c>
+      <c r="F5" s="14">
+        <v>3000</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="17">
-        <v>5000</v>
-      </c>
-      <c r="C6" s="17">
-        <v>0</v>
-      </c>
-      <c r="D6" s="17">
-        <v>0</v>
-      </c>
-      <c r="E6" s="17">
-        <v>0</v>
-      </c>
-      <c r="F6" s="17">
-        <v>5000</v>
+        <v>34</v>
+      </c>
+      <c r="B6" s="14">
+        <v>9000</v>
+      </c>
+      <c r="C6" s="14">
+        <v>0</v>
+      </c>
+      <c r="D6" s="14">
+        <v>0</v>
+      </c>
+      <c r="E6" s="14">
+        <v>0</v>
+      </c>
+      <c r="F6" s="14">
+        <v>9000</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="17">
-        <v>7000</v>
-      </c>
-      <c r="C7" s="17">
-        <v>1000</v>
-      </c>
-      <c r="D7" s="17">
-        <v>0</v>
-      </c>
-      <c r="E7" s="17">
-        <v>0</v>
-      </c>
-      <c r="F7" s="17">
-        <v>8000</v>
+        <v>35</v>
+      </c>
+      <c r="B7" s="14">
+        <v>13000</v>
+      </c>
+      <c r="C7" s="14">
+        <v>0</v>
+      </c>
+      <c r="D7" s="14">
+        <v>0</v>
+      </c>
+      <c r="E7" s="14">
+        <v>0</v>
+      </c>
+      <c r="F7" s="14">
+        <v>13000</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="17">
+        <v>36</v>
+      </c>
+      <c r="B8" s="14">
+        <v>16000</v>
+      </c>
+      <c r="C8" s="14">
         <v>10000</v>
       </c>
-      <c r="C8" s="17">
-        <v>8000</v>
-      </c>
-      <c r="D8" s="17">
-        <v>0</v>
-      </c>
-      <c r="E8" s="17">
-        <v>0</v>
-      </c>
-      <c r="F8" s="17">
-        <v>18000</v>
+      <c r="D8" s="14">
+        <v>0</v>
+      </c>
+      <c r="E8" s="14">
+        <v>0</v>
+      </c>
+      <c r="F8" s="14">
+        <v>26000</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="17">
-        <v>15000</v>
-      </c>
-      <c r="C9" s="17">
-        <v>14000</v>
-      </c>
-      <c r="D9" s="17">
-        <v>0</v>
-      </c>
-      <c r="E9" s="17">
-        <v>0</v>
-      </c>
-      <c r="F9" s="17">
-        <v>29000</v>
+        <v>37</v>
+      </c>
+      <c r="B9" s="14">
+        <v>20000</v>
+      </c>
+      <c r="C9" s="14">
+        <v>24000</v>
+      </c>
+      <c r="D9" s="14">
+        <v>0</v>
+      </c>
+      <c r="E9" s="14">
+        <v>0</v>
+      </c>
+      <c r="F9" s="14">
+        <v>44000</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="17">
-        <v>19000</v>
-      </c>
-      <c r="C10" s="17">
-        <v>19000</v>
-      </c>
-      <c r="D10" s="17">
-        <v>2000</v>
-      </c>
-      <c r="E10" s="17">
-        <v>0</v>
-      </c>
-      <c r="F10" s="17">
-        <v>39000</v>
+        <v>38</v>
+      </c>
+      <c r="B10" s="14">
+        <v>23000</v>
+      </c>
+      <c r="C10" s="14">
+        <v>33000</v>
+      </c>
+      <c r="D10" s="14">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="14">
+        <v>0</v>
+      </c>
+      <c r="F10" s="14">
+        <v>57000</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="17">
-        <v>20000</v>
-      </c>
-      <c r="C11" s="17">
-        <v>27000</v>
-      </c>
-      <c r="D11" s="17">
-        <v>11000</v>
-      </c>
-      <c r="E11" s="17">
-        <v>0</v>
-      </c>
-      <c r="F11" s="17">
-        <v>58000</v>
+        <v>39</v>
+      </c>
+      <c r="B11" s="14">
+        <v>24000</v>
+      </c>
+      <c r="C11" s="14">
+        <v>41000</v>
+      </c>
+      <c r="D11" s="14">
+        <v>10000</v>
+      </c>
+      <c r="E11" s="14">
+        <v>0</v>
+      </c>
+      <c r="F11" s="14">
+        <v>74000</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="17">
-        <v>20000</v>
-      </c>
-      <c r="C12" s="17">
-        <v>37000</v>
-      </c>
-      <c r="D12" s="17">
-        <v>20000</v>
-      </c>
-      <c r="E12" s="17">
-        <v>0</v>
-      </c>
-      <c r="F12" s="17">
-        <v>77000</v>
+        <v>40</v>
+      </c>
+      <c r="B12" s="14">
+        <v>25000</v>
+      </c>
+      <c r="C12" s="14">
+        <v>50000</v>
+      </c>
+      <c r="D12" s="14">
+        <v>29000</v>
+      </c>
+      <c r="E12" s="14">
+        <v>0</v>
+      </c>
+      <c r="F12" s="14">
+        <v>104000</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="17">
-        <v>26000</v>
-      </c>
-      <c r="C13" s="17">
-        <v>45000</v>
-      </c>
-      <c r="D13" s="17">
-        <v>26000</v>
-      </c>
-      <c r="E13" s="17">
-        <v>0</v>
-      </c>
-      <c r="F13" s="17">
-        <v>98000</v>
+        <v>41</v>
+      </c>
+      <c r="B13" s="14">
+        <v>28000</v>
+      </c>
+      <c r="C13" s="14">
+        <v>58000</v>
+      </c>
+      <c r="D13" s="14">
+        <v>44000</v>
+      </c>
+      <c r="E13" s="14">
+        <v>0</v>
+      </c>
+      <c r="F13" s="14">
+        <v>130000</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" s="17">
-        <v>28000</v>
-      </c>
-      <c r="C14" s="17">
-        <v>47000</v>
-      </c>
-      <c r="D14" s="17">
-        <v>33000</v>
-      </c>
-      <c r="E14" s="17">
-        <v>1000</v>
-      </c>
-      <c r="F14" s="17">
-        <v>110000</v>
+        <v>42</v>
+      </c>
+      <c r="B14" s="14">
+        <v>31000</v>
+      </c>
+      <c r="C14" s="14">
+        <v>57000</v>
+      </c>
+      <c r="D14" s="14">
+        <v>53000</v>
+      </c>
+      <c r="E14" s="14">
+        <v>2000</v>
+      </c>
+      <c r="F14" s="14">
+        <v>143000</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15" s="17">
-        <v>30000</v>
-      </c>
-      <c r="C15" s="17">
-        <v>50000</v>
-      </c>
-      <c r="D15" s="17">
-        <v>58000</v>
-      </c>
-      <c r="E15" s="17">
-        <v>3000</v>
-      </c>
-      <c r="F15" s="17">
-        <v>141000</v>
+        <v>43</v>
+      </c>
+      <c r="B15" s="14">
+        <v>36000</v>
+      </c>
+      <c r="C15" s="14">
+        <v>63000</v>
+      </c>
+      <c r="D15" s="14">
+        <v>76000</v>
+      </c>
+      <c r="E15" s="14">
+        <v>5000</v>
+      </c>
+      <c r="F15" s="14">
+        <v>180000</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B16" s="3">
-        <v>183000</v>
+        <v>227000</v>
       </c>
       <c r="C16" s="3">
-        <v>250000</v>
+        <v>336000</v>
       </c>
       <c r="D16" s="3">
-        <v>149000</v>
+        <v>214000</v>
       </c>
       <c r="E16" s="3">
-        <v>4000</v>
+        <v>7000</v>
       </c>
       <c r="F16" s="3">
-        <v>587000</v>
+        <v>784000</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
-        <v>36</v>
+      <c r="A18" s="15" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1189,192 +1336,207 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>42</v>
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="6">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="7">
-        <v>2</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" s="10">
+      <c r="E4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="7">
-        <v>12</v>
-      </c>
-      <c r="E5" s="7">
-        <v>1</v>
-      </c>
-      <c r="F5" s="10">
-        <v>7000</v>
+        <v>53</v>
+      </c>
+      <c r="D5" s="6">
+        <v>27</v>
+      </c>
+      <c r="E5" s="6">
+        <v>2</v>
+      </c>
+      <c r="F5" s="8">
+        <v>178000</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="7">
-        <v>21</v>
-      </c>
-      <c r="E6" s="7">
+        <v>53</v>
+      </c>
+      <c r="D6" s="6">
+        <v>30</v>
+      </c>
+      <c r="E6" s="6">
         <v>1</v>
       </c>
-      <c r="F6" s="10">
-        <v>20000</v>
+      <c r="F6" s="8">
+        <v>6000</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="7">
-        <v>1</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="10">
+        <v>53</v>
+      </c>
+      <c r="D7" s="6">
+        <v>4</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F7" s="8">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>52</v>
+      <c r="A10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="E11" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="17">
-        <v>7000</v>
+        <v>65</v>
+      </c>
+      <c r="F11" s="14">
+        <v>66000</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="E12" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="17">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
-        <v>60</v>
+        <v>65</v>
+      </c>
+      <c r="F12" s="14">
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E13" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" s="14">
+        <v>6000</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
-        <v>61</v>
+      <c r="A15" s="15" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>62</v>
+      <c r="A16" s="15" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>63</v>
+      <c r="A17" s="15" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1397,60 +1559,60 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>65</v>
+      <c r="A3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="4">
-        <v>106.9</v>
+        <v>9</v>
+      </c>
+      <c r="B4" s="13">
+        <v>96.3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="4">
-        <v>271.5</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="13">
+        <v>234.3</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="4">
-        <v>525</v>
+        <v>13</v>
+      </c>
+      <c r="B6" s="13">
+        <v>522</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="4">
-        <v>53.9</v>
+        <v>15</v>
+      </c>
+      <c r="B7" s="13">
+        <v>54.9</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="18">
-        <v>957.3</v>
+        <v>17</v>
+      </c>
+      <c r="B8" s="16">
+        <v>907.5</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1464,7 +1626,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -1473,87 +1635,79 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>68</v>
+      <c r="A3" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>70</v>
+      <c r="A4" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
-        <v>73</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
-        <v>77</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>80</v>
+      <c r="A5" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>82</v>
+      <c r="A10" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>86</v>
+      <c r="A11" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PAUSED (task130): rule 3 rework 3b (second layer), stage 3 green
Round 3b adds a second analytical layer: the Early Resolution Program's
disclosure settlements began at each entity between January and July 2019
(none before, steady after), so the 2027 window is costed on each entity's
experience from its first settlement, each Claim at its own report lag.
Call $1,250,000 ($1,281,536, SE $65,916); the loss-weighted step factor on
the whole 2016 to 2024 experience files $1,000,000 ($961,261, 1.28 bins).
Funding policy 3.1 files the estimand as Claims as they will arise and be
made in the Plan Year; 3.3 states the experience the trust holds; claims
seed 3006. Resume at stage 4: a fresh reader and judge.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task130/golden/trust_funding_2027.xlsx
+++ b/task130/golden/trust_funding_2027.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="134">
   <si>
     <t>Corvane Professional Liability Trust: 2027 contribution</t>
   </si>
@@ -48,40 +48,97 @@
     <t>Months in the Trust in 2027</t>
   </si>
   <si>
+    <t>Experience used from</t>
+  </si>
+  <si>
     <t>Tolliver Falls Hospital</t>
   </si>
   <si>
     <t>1 January 2027</t>
   </si>
   <si>
+    <t>April 2019</t>
+  </si>
+  <si>
     <t>Alderwick Medical Center</t>
   </si>
   <si>
     <t>1 April 2027</t>
   </si>
   <si>
+    <t>January 2019</t>
+  </si>
+  <si>
     <t>Corvane Medical Group</t>
   </si>
   <si>
     <t>1 July 2027</t>
   </si>
   <si>
+    <t>May 2019</t>
+  </si>
+  <si>
     <t>Brennick Community Hospital</t>
   </si>
   <si>
     <t>1 October 2027</t>
   </si>
   <si>
+    <t>July 2019</t>
+  </si>
+  <si>
     <t>Experience</t>
   </si>
   <si>
-    <t>Claims from 2016 to 2024 incidents naming Covered Clinicians</t>
+    <t>Claims from 2016 to 2024 incidents naming Covered Clinicians (held by the Trust)</t>
   </si>
   <si>
     <t>Covered FTE-years, 2016 to 2024 payroll</t>
   </si>
   <si>
-    <t>Experience Claims by delay from incident to first making</t>
+    <t>Claims used: incidents from each entity's first disclosure settlement to December 2024</t>
+  </si>
+  <si>
+    <t>Covered FTE-years over the same months</t>
+  </si>
+  <si>
+    <t>Claims made within 30 days of the incident, by incident year</t>
+  </si>
+  <si>
+    <t>Incident year</t>
+  </si>
+  <si>
+    <t>All entities</t>
+  </si>
+  <si>
+    <t>2016</t>
+  </si>
+  <si>
+    <t>2017</t>
+  </si>
+  <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>2019</t>
+  </si>
+  <si>
+    <t>2020</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>2023</t>
+  </si>
+  <si>
+    <t>2024</t>
+  </si>
+  <si>
+    <t>Experience used, by delay from incident to first making</t>
   </si>
   <si>
     <t>Delay</t>
@@ -108,7 +165,10 @@
     <t>A year or more</t>
   </si>
   <si>
-    <t>Only Claims made by 31 December 2027 from incidents on or after each entity's Transition Date fall in 2027. In the experience the Claims made within weeks of the care are disclosed harm settled through the Early Resolution Program, those made in the following months mostly small program requests, and the cost sits in the demands and suits made a year or more after the care.</t>
+    <t>Only Claims made by 31 December 2027 from incidents on or after each entity's Transition Date fall in 2027. In the experience the Claims made within weeks of the care are harm the care team disclosed and the Early Resolution Program settled, those made in the following months mostly small program requests, and the cost sits in the demands and suits made a year or more after the care.</t>
+  </si>
+  <si>
+    <t>The disclosure settlements begin at each entity in 2019 and run in every year since; no 2016 to 2018 incident has one. The 2027 window is costed on each entity's experience from the month of its first settlement, the claims process 2027 will have; the whole 2016 to 2024 experience would give $1,000,000.</t>
   </si>
   <si>
     <t>Source: risk management claims register extract valued 30 September 2026; legacy payroll 2016 to 2024; clinician staffing plan 2027, version 2026-09-29. Definitions on the Notes sheet.</t>
@@ -144,21 +204,21 @@
     <t>valued 30 September 2026</t>
   </si>
   <si>
+    <t>1 April 2019</t>
+  </si>
+  <si>
+    <t>Stoneleigh Casualty Insurance Company</t>
+  </si>
+  <si>
+    <t>1 July 2019</t>
+  </si>
+  <si>
+    <t>1 October 2022</t>
+  </si>
+  <si>
     <t>None</t>
   </si>
   <si>
-    <t>1 April 2019</t>
-  </si>
-  <si>
-    <t>Stoneleigh Casualty Insurance Company</t>
-  </si>
-  <si>
-    <t>1 July 2019</t>
-  </si>
-  <si>
-    <t>1 October 2022</t>
-  </si>
-  <si>
     <t>Claims missing from the loss runs</t>
   </si>
   <si>
@@ -180,105 +240,99 @@
     <t>Our reserves ($)</t>
   </si>
   <si>
-    <t>CL-2026-1143</t>
-  </si>
-  <si>
-    <t>IR-2025-01259</t>
-  </si>
-  <si>
-    <t>7 Feb 2025</t>
-  </si>
-  <si>
-    <t>25 Sep 2026</t>
+    <t>CL-2026-1051</t>
+  </si>
+  <si>
+    <t>IR-2026-07136</t>
+  </si>
+  <si>
+    <t>13 Dec 2023</t>
+  </si>
+  <si>
+    <t>28 Sep 2026</t>
   </si>
   <si>
     <t>Claim</t>
   </si>
   <si>
-    <t>CL-2026-1140</t>
-  </si>
-  <si>
-    <t>IR-2025-09682</t>
-  </si>
-  <si>
-    <t>8 Dec 2025</t>
+    <t>CL-2026-1065</t>
+  </si>
+  <si>
+    <t>IR-2026-00555</t>
+  </si>
+  <si>
+    <t>8 Jan 2026</t>
+  </si>
+  <si>
+    <t>30 Sep 2026</t>
+  </si>
+  <si>
+    <t>CL-2026-0931</t>
+  </si>
+  <si>
+    <t>IR-2026-02574</t>
+  </si>
+  <si>
+    <t>23 Mar 2026</t>
+  </si>
+  <si>
+    <t>21 Aug 2026</t>
+  </si>
+  <si>
+    <t>CL-2026-1056</t>
+  </si>
+  <si>
+    <t>IR-2026-04894</t>
+  </si>
+  <si>
+    <t>24 Jun 2026</t>
+  </si>
+  <si>
+    <t>CL-2026-0823</t>
+  </si>
+  <si>
+    <t>IR-2025-08954</t>
+  </si>
+  <si>
+    <t>10 Nov 2025</t>
+  </si>
+  <si>
+    <t>21 Jul 2026</t>
+  </si>
+  <si>
+    <t>CL-2026-1050</t>
+  </si>
+  <si>
+    <t>IR-2026-01782</t>
+  </si>
+  <si>
+    <t>27 Feb 2026</t>
   </si>
   <si>
     <t>24 Sep 2026</t>
   </si>
   <si>
-    <t>CL-2026-0833</t>
-  </si>
-  <si>
-    <t>IR-2026-00766</t>
-  </si>
-  <si>
-    <t>29 Jan 2026</t>
-  </si>
-  <si>
-    <t>2 Jul 2026</t>
-  </si>
-  <si>
-    <t>CL-2026-1161</t>
-  </si>
-  <si>
-    <t>IR-2026-02619</t>
-  </si>
-  <si>
-    <t>23 Apr 2026</t>
+    <t>CL-2026-1061</t>
+  </si>
+  <si>
+    <t>IR-2026-07157</t>
+  </si>
+  <si>
+    <t>18 Aug 2026</t>
+  </si>
+  <si>
+    <t>CL-2026-1063</t>
+  </si>
+  <si>
+    <t>IR-2026-07201</t>
+  </si>
+  <si>
+    <t>14 Sep 2026</t>
   </si>
   <si>
     <t>29 Sep 2026</t>
   </si>
   <si>
-    <t>CL-2026-0952</t>
-  </si>
-  <si>
-    <t>IR-2025-06129</t>
-  </si>
-  <si>
-    <t>15 Aug 2025</t>
-  </si>
-  <si>
-    <t>4 Aug 2026</t>
-  </si>
-  <si>
-    <t>CL-2026-1148</t>
-  </si>
-  <si>
-    <t>IR-2025-07789</t>
-  </si>
-  <si>
-    <t>26 Sep 2025</t>
-  </si>
-  <si>
-    <t>CL-2026-1157</t>
-  </si>
-  <si>
-    <t>IR-2026-00820</t>
-  </si>
-  <si>
-    <t>27 Jan 2026</t>
-  </si>
-  <si>
-    <t>CL-2026-1141</t>
-  </si>
-  <si>
-    <t>IR-2026-01373</t>
-  </si>
-  <si>
-    <t>17 Feb 2026</t>
-  </si>
-  <si>
-    <t>CL-2026-1151</t>
-  </si>
-  <si>
-    <t>IR-2026-02011</t>
-  </si>
-  <si>
-    <t>19 Mar 2026</t>
-  </si>
-  <si>
     <t>Each expiring carrier's policies are the terms it wrote for the entity, from the date in the premium history; open claims from incidents before that date are under the former carrier's occurrence policies (trust agreement 2.2), so they are not looked for on these runs.</t>
   </si>
   <si>
@@ -303,9 +357,6 @@
     <t>September 2026</t>
   </si>
   <si>
-    <t>All entities</t>
-  </si>
-  <si>
     <t>Paid FTE: the hours paid on each covered position's pay lines in the work month (regular and paid time off) over the 173.33 hours scheduled a month at 1.0 FTE; a per-diem clinician by the shifts paid, a month of unpaid leave at none.</t>
   </si>
   <si>
@@ -336,7 +387,13 @@
     <t>Each entity from its Transition Date (its Retroactive Date) to 31 December 2027: Claims made in 2027 from incidents on or after that date.</t>
   </si>
   <si>
-    <t>The 3,043 Claims from incidents in 2016 to 2024 naming Covered Clinicians, valued at paid plus case reserves on the Covered Clinicians' rows of the register extract valued 30 September 2026 and trended at 5.0% a year from the incident year to 2027, against 13,747.1 covered FTE-years in the payroll for the same years, pooled within each specialty class (funding policy 3.2 to 3.4).</t>
+    <t>The 2,288 Claims from incidents naming Covered Clinicians from each entity's first disclosure settlement (Tolliver Falls Hospital April 2019, Alderwick Medical Center January 2019, Corvane Medical Group May 2019, Brennick Community Hospital July 2019) to December 2024, valued at paid plus case reserves on the Covered Clinicians' rows of the register extract valued 30 September 2026 and trended at 5.0% a year from the incident year to 2027, against 9,330.0 covered FTE-years in the payroll for the same entities and months, by specialty class (funding policy 3.2 to 3.4). The Trust holds 3,320 Claims from 2016 to 2024 on 13,747.1 FTE-years (3.3).</t>
+  </si>
+  <si>
+    <t>Experience period</t>
+  </si>
+  <si>
+    <t>A disclosure settlement is a Claim made within 30 days of its incident; none is made from an incident before each entity's month above, and they run in every year since. The 2027 Claims will be made under this claims process (funding policy 3.1), so the months before it are left out. Every delay the 2027 window can use (under a year) is complete in the extract for every incident to December 2024.</t>
   </si>
   <si>
     <t>Exposure</t>
@@ -776,26 +833,28 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="58.7109375" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" customWidth="1"/>
-    <col min="4" max="4" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="24.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.7109375" customWidth="1"/>
+    <col min="5" max="5" width="24.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -806,12 +865,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>5</v>
       </c>
@@ -821,155 +880,396 @@
       <c r="C7" s="6" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D8" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C9">
         <v>9</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C10">
         <v>6</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C11">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D11" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C14" s="8">
-        <v>3043</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3320</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C15" s="9">
         <v>13747.1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="6" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="8">
+        <v>2288</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="9">
+        <v>9330</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="8">
+        <v>0</v>
+      </c>
+      <c r="C21" s="8">
+        <v>0</v>
+      </c>
+      <c r="D21" s="8">
+        <v>0</v>
+      </c>
+      <c r="E21" s="8">
+        <v>0</v>
+      </c>
+      <c r="F21" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="8">
+        <v>0</v>
+      </c>
+      <c r="C22" s="8">
+        <v>0</v>
+      </c>
+      <c r="D22" s="8">
+        <v>0</v>
+      </c>
+      <c r="E22" s="8">
+        <v>0</v>
+      </c>
+      <c r="F22" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="8">
+        <v>0</v>
+      </c>
+      <c r="C23" s="8">
+        <v>0</v>
+      </c>
+      <c r="D23" s="8">
+        <v>0</v>
+      </c>
+      <c r="E23" s="8">
+        <v>0</v>
+      </c>
+      <c r="F23" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="8">
+        <v>5</v>
+      </c>
+      <c r="C24" s="8">
         <v>23</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>24</v>
-      </c>
-      <c r="B19" s="8">
-        <v>208</v>
-      </c>
-      <c r="C19" s="8">
-        <v>55000</v>
-      </c>
-      <c r="D19" s="10">
-        <v>0.07207586355158489</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="D24" s="8">
+        <v>14</v>
+      </c>
+      <c r="E24" s="8">
+        <v>3</v>
+      </c>
+      <c r="F24" s="8">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="8">
+        <v>8</v>
+      </c>
+      <c r="C25" s="8">
+        <v>15</v>
+      </c>
+      <c r="D25" s="8">
+        <v>26</v>
+      </c>
+      <c r="E25" s="8">
+        <v>0</v>
+      </c>
+      <c r="F25" s="8">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="8">
+        <v>9</v>
+      </c>
+      <c r="C26" s="8">
+        <v>11</v>
+      </c>
+      <c r="D26" s="8">
+        <v>16</v>
+      </c>
+      <c r="E26" s="8">
+        <v>4</v>
+      </c>
+      <c r="F26" s="8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" s="8">
+        <v>9</v>
+      </c>
+      <c r="C27" s="8">
+        <v>17</v>
+      </c>
+      <c r="D27" s="8">
+        <v>37</v>
+      </c>
+      <c r="E27" s="8">
+        <v>1</v>
+      </c>
+      <c r="F27" s="8">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" s="8">
+        <v>2</v>
+      </c>
+      <c r="C28" s="8">
+        <v>15</v>
+      </c>
+      <c r="D28" s="8">
         <v>25</v>
       </c>
-      <c r="B20" s="8">
+      <c r="E28" s="8">
+        <v>5</v>
+      </c>
+      <c r="F28" s="8">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" s="8">
+        <v>8</v>
+      </c>
+      <c r="C29" s="8">
+        <v>15</v>
+      </c>
+      <c r="D29" s="8">
+        <v>23</v>
+      </c>
+      <c r="E29" s="8">
+        <v>4</v>
+      </c>
+      <c r="F29" s="8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="8">
+        <v>295</v>
+      </c>
+      <c r="C33" s="8">
+        <v>28000</v>
+      </c>
+      <c r="D33" s="10">
+        <v>0.07999674318772448</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="8">
+        <v>38</v>
+      </c>
+      <c r="C34" s="8">
+        <v>17000</v>
+      </c>
+      <c r="D34" s="10">
+        <v>0.006352909074798874</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" s="8">
+        <v>1768</v>
+      </c>
+      <c r="C35" s="8">
+        <v>9000</v>
+      </c>
+      <c r="D35" s="10">
+        <v>0.1577367086764098</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="8">
-        <v>39000</v>
-      </c>
-      <c r="D20" s="10">
-        <v>0.01143105903041128</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="8">
-        <v>2512</v>
-      </c>
-      <c r="C21" s="8">
-        <v>9000</v>
-      </c>
-      <c r="D21" s="10">
-        <v>0.1375763289544716</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>27</v>
-      </c>
-      <c r="B22" s="8">
-        <v>277</v>
-      </c>
-      <c r="C22" s="8">
-        <v>443000</v>
-      </c>
-      <c r="D22" s="10">
-        <v>0.7789167484635322</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>29</v>
+      <c r="B36" s="8">
+        <v>187</v>
+      </c>
+      <c r="C36" s="8">
+        <v>421000</v>
+      </c>
+      <c r="D36" s="10">
+        <v>0.7559136390610669</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -983,7 +1283,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.7109375" customWidth="1"/>
@@ -997,7 +1297,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1005,111 +1305,111 @@
         <v>5</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="E4" s="7">
-        <v>21</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>40</v>
+        <v>16</v>
+      </c>
+      <c r="F4" s="7">
+        <v>1</v>
       </c>
       <c r="G4" s="11">
-        <v>0</v>
+        <v>1465000</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="E5" s="7">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="F5" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G5" s="11">
-        <v>839000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="E6" s="7">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="F6" s="7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G6" s="11">
-        <v>16000</v>
+        <v>54000</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="E7" s="7">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="G7" s="11">
         <v>0</v>
@@ -1117,7 +1417,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1125,88 +1425,88 @@
         <v>5</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="D11" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="E11" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G11" s="8">
-        <v>832000</v>
+        <v>1465000</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F12" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G12" s="8">
-        <v>5000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="D13" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G13" s="8">
         <v>0</v>
@@ -1214,160 +1514,137 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="C14" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="D14" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="E14" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="F14" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G14" s="8">
-        <v>2000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="C15" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="D15" t="s">
-        <v>71</v>
+        <v>90</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="F15" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G15" s="8">
-        <v>3000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="C16" t="s">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E16" t="s">
-        <v>55</v>
+        <v>95</v>
       </c>
       <c r="F16" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G16" s="8">
-        <v>2000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B17" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" t="s">
         <v>76</v>
       </c>
-      <c r="C17" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" t="s">
-        <v>78</v>
-      </c>
-      <c r="E17" t="s">
-        <v>68</v>
-      </c>
-      <c r="F17" t="s">
-        <v>56</v>
-      </c>
       <c r="G17" s="8">
-        <v>8000</v>
+        <v>24000</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D18" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>102</v>
       </c>
       <c r="F18" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="G18" s="8">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" t="s">
-        <v>84</v>
-      </c>
-      <c r="E19" t="s">
-        <v>55</v>
-      </c>
-      <c r="F19" t="s">
-        <v>56</v>
-      </c>
-      <c r="G19" s="8">
-        <v>1000</v>
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>86</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>88</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1392,7 +1669,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1400,18 +1677,18 @@
         <v>5</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="9">
         <v>188.6</v>
@@ -1425,7 +1702,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B5" s="9">
         <v>464.5</v>
@@ -1439,7 +1716,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B6" s="9">
         <v>1037.1</v>
@@ -1453,7 +1730,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B7" s="9">
         <v>105.5</v>
@@ -1467,7 +1744,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="B8" s="13">
         <v>1795.8</v>
@@ -1481,22 +1758,22 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>94</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>95</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>96</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -1510,7 +1787,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
@@ -1519,79 +1796,87 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>101</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>102</v>
+        <v>119</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>114</v>
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>